<commit_message>
added hdd,ssd,m2ssd and motherboard support
</commit_message>
<xml_diff>
--- a/docs/partpicker_db_plan.xlsx
+++ b/docs/partpicker_db_plan.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="38" uniqueCount="38">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="46" uniqueCount="46">
   <si>
     <t xml:space="preserve">pcpartpicker sqlite db</t>
   </si>
@@ -108,6 +108,18 @@
     <t>formFactorID</t>
   </si>
   <si>
+    <t>ramSlots</t>
+  </si>
+  <si>
+    <t>pcieSlots</t>
+  </si>
+  <si>
+    <t>sataSlots</t>
+  </si>
+  <si>
+    <t>m2Slots</t>
+  </si>
+  <si>
     <t>PSU</t>
   </si>
   <si>
@@ -130,6 +142,18 @@
   </si>
   <si>
     <t>fanSlots</t>
+  </si>
+  <si>
+    <t>SSD</t>
+  </si>
+  <si>
+    <t>M2SSD</t>
+  </si>
+  <si>
+    <t>HDD</t>
+  </si>
+  <si>
+    <t>User</t>
   </si>
 </sst>
 </file>
@@ -206,7 +230,7 @@
   <cellStyleXfs count="1">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="12">
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0"/>
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1"/>
     <xf fontId="0" fillId="0" borderId="2" numFmtId="0" xfId="0" applyBorder="1"/>
@@ -216,24 +240,23 @@
     <xf fontId="0" fillId="0" borderId="1" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
+    <xf fontId="0" fillId="0" borderId="2" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="2" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf fontId="0" fillId="0" borderId="3" numFmtId="0" xfId="0" applyBorder="1"/>
+    <xf fontId="0" fillId="0" borderId="4" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf fontId="0" fillId="0" borderId="0" numFmtId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="2" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf fontId="0" fillId="0" borderId="3" numFmtId="0" xfId="0" applyBorder="1"/>
-    <xf fontId="0" fillId="0" borderId="3" numFmtId="0" xfId="0" applyBorder="1"/>
     <xf fontId="0" fillId="0" borderId="4" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf fontId="0" fillId="0" borderId="4" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf fontId="0" fillId="0" borderId="3" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf fontId="0" fillId="0" borderId="3" numFmtId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -752,8 +775,8 @@
       <c r="F1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="G1" s="5"/>
-      <c r="H1" s="6"/>
+      <c r="G1" s="3"/>
+      <c r="H1" s="5"/>
     </row>
     <row r="3" ht="14.25">
       <c r="A3" s="3" t="s">
@@ -764,114 +787,114 @@
       <c r="F3" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="7"/>
-      <c r="H3" s="8"/>
+      <c r="G3" s="3"/>
+      <c r="H3" s="5"/>
     </row>
     <row r="4" ht="14.25">
-      <c r="A4" s="9" t="s">
+      <c r="A4" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="9" t="s">
+      <c r="B4" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="C4" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="F4" s="9" t="s">
+      <c r="C4" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F4" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="G4" s="9" t="s">
+      <c r="G4" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="H4" s="9" t="s">
+      <c r="H4" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="5" ht="14.25">
-      <c r="A5" s="9" t="s">
+      <c r="A5" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="B5" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="C5" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="F5" s="9" t="s">
+      <c r="B5" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F5" s="6" t="s">
         <v>9</v>
       </c>
-      <c r="G5" s="9"/>
-      <c r="H5" s="9" t="s">
+      <c r="G5" s="6"/>
+      <c r="H5" s="6" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="6" ht="14.25">
-      <c r="A6" s="9" t="s">
+      <c r="A6" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B6" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="C6" s="9" t="s">
+      <c r="B6" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="7" ht="14.25">
-      <c r="A7" s="9" t="s">
+      <c r="A7" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B7" s="9"/>
-      <c r="C7" s="9" t="s">
+      <c r="B7" s="6"/>
+      <c r="C7" s="6" t="s">
         <v>13</v>
       </c>
       <c r="F7" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="G7" s="7"/>
-      <c r="H7" s="8"/>
+      <c r="G7" s="3"/>
+      <c r="H7" s="5"/>
     </row>
     <row r="8" ht="14.25">
-      <c r="A8" s="9" t="s">
+      <c r="A8" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B8" s="9"/>
-      <c r="C8" s="9" t="s">
+      <c r="B8" s="6"/>
+      <c r="C8" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="F8" s="9" t="s">
+      <c r="F8" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="G8" s="9" t="s">
+      <c r="G8" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="H8" s="9" t="s">
+      <c r="H8" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="9" ht="14.25">
-      <c r="A9" s="9" t="s">
+      <c r="A9" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B9" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="C9" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="F9" s="10" t="s">
+      <c r="B9" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C9" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F9" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="G9" s="9"/>
-      <c r="H9" s="9" t="s">
+      <c r="G9" s="6"/>
+      <c r="H9" s="6" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="10" ht="14.25">
-      <c r="A10" s="9" t="s">
+      <c r="A10" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="B10" s="9"/>
-      <c r="C10" s="9" t="s">
+      <c r="B10" s="6"/>
+      <c r="C10" s="6" t="s">
         <v>6</v>
       </c>
     </row>
@@ -879,8 +902,8 @@
       <c r="F11" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="G11" s="5"/>
-      <c r="H11" s="6"/>
+      <c r="G11" s="3"/>
+      <c r="H11" s="5"/>
     </row>
     <row r="12" ht="14.25">
       <c r="A12" s="3" t="s">
@@ -888,470 +911,734 @@
       </c>
       <c r="B12" s="3"/>
       <c r="C12" s="3"/>
-      <c r="F12" s="9" t="s">
+      <c r="F12" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="G12" s="9" t="s">
+      <c r="G12" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="H12" s="9" t="s">
+      <c r="H12" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="13" ht="14.25">
-      <c r="A13" s="9" t="s">
+      <c r="A13" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="B13" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="C13" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="F13" s="9" t="s">
+      <c r="C13" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F13" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="G13" s="9"/>
-      <c r="H13" s="9" t="s">
+      <c r="G13" s="6"/>
+      <c r="H13" s="6" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="14" ht="14.25">
-      <c r="A14" s="9" t="s">
+      <c r="A14" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B14" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="C14" s="9" t="s">
+      <c r="B14" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C14" s="6" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="15" ht="14.25">
-      <c r="A15" s="9" t="s">
+      <c r="A15" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B15" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="C15" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="F15" s="7" t="s">
+      <c r="B15" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C15" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F15" s="3" t="s">
         <v>21</v>
       </c>
-      <c r="G15" s="5"/>
-      <c r="H15" s="5"/>
+      <c r="G15" s="3"/>
+      <c r="H15" s="3"/>
     </row>
     <row r="16" ht="14.25">
-      <c r="A16" s="9" t="s">
+      <c r="A16" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B16" s="9"/>
-      <c r="C16" s="9" t="s">
-        <v>13</v>
-      </c>
-      <c r="F16" s="9" t="s">
+      <c r="B16" s="6"/>
+      <c r="C16" s="6" t="s">
+        <v>13</v>
+      </c>
+      <c r="F16" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="G16" s="9" t="s">
+      <c r="G16" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="H16" s="9" t="s">
+      <c r="H16" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="17" ht="14.25">
-      <c r="A17" s="9" t="s">
+      <c r="A17" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B17" s="9"/>
-      <c r="C17" s="9" t="s">
+      <c r="B17" s="6"/>
+      <c r="C17" s="6" t="s">
         <v>16</v>
       </c>
-      <c r="F17" s="9" t="s">
+      <c r="F17" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="G17" s="9"/>
-      <c r="H17" s="9" t="s">
+      <c r="G17" s="6"/>
+      <c r="H17" s="6" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="18" ht="14.25">
-      <c r="A18" s="9" t="s">
+      <c r="A18" s="6" t="s">
         <v>22</v>
       </c>
-      <c r="B18" s="9"/>
-      <c r="C18" s="9" t="s">
+      <c r="B18" s="6"/>
+      <c r="C18" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="19" ht="14.25">
-      <c r="F19" s="11" t="s">
+      <c r="F19" s="7" t="s">
         <v>23</v>
       </c>
-      <c r="G19" s="12"/>
-      <c r="H19" s="12"/>
+      <c r="G19" s="7"/>
+      <c r="H19" s="7"/>
     </row>
     <row r="20" ht="14.25">
-      <c r="A20" s="7" t="s">
+      <c r="A20" s="3" t="s">
         <v>24</v>
       </c>
-      <c r="B20" s="5"/>
-      <c r="C20" s="5"/>
-      <c r="F20" s="9" t="s">
+      <c r="B20" s="3"/>
+      <c r="C20" s="3"/>
+      <c r="F20" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="G20" s="9" t="s">
+      <c r="G20" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="H20" s="9" t="s">
+      <c r="H20" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="21" ht="14.25">
-      <c r="A21" s="9" t="s">
+      <c r="A21" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B21" s="9" t="s">
+      <c r="B21" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="C21" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="F21" s="9" t="s">
+      <c r="C21" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="F21" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="G21" s="9"/>
-      <c r="H21" s="9" t="s">
+      <c r="G21" s="6"/>
+      <c r="H21" s="6" t="s">
         <v>10</v>
       </c>
     </row>
     <row r="22" ht="14.25">
-      <c r="A22" s="9" t="s">
+      <c r="A22" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B22" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="C22" s="9" t="s">
+      <c r="B22" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C22" s="6" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="23" ht="14.25">
-      <c r="A23" s="9" t="s">
+      <c r="A23" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B23" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="C23" s="9" t="s">
+      <c r="B23" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C23" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="24" ht="14.25">
-      <c r="A24" s="9" t="s">
+      <c r="A24" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B24" s="9"/>
-      <c r="C24" s="9" t="s">
+      <c r="B24" s="6"/>
+      <c r="C24" s="6" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="25" ht="14.25">
-      <c r="A25" s="9" t="s">
+      <c r="A25" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B25" s="9"/>
-      <c r="C25" s="9" t="s">
+      <c r="B25" s="6"/>
+      <c r="C25" s="6" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="26" ht="14.25">
-      <c r="A26" s="9" t="s">
+      <c r="A26" s="6" t="s">
         <v>25</v>
       </c>
-      <c r="B26" s="9"/>
-      <c r="C26" s="9" t="s">
+      <c r="B26" s="6"/>
+      <c r="C26" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="27" ht="14.25">
-      <c r="A27" s="9" t="s">
+      <c r="A27" s="6" t="s">
         <v>26</v>
       </c>
-      <c r="B27" s="9"/>
-      <c r="C27" s="9" t="s">
+      <c r="B27" s="6"/>
+      <c r="C27" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="28" ht="14.25">
-      <c r="A28" s="9" t="s">
+      <c r="A28" s="6" t="s">
         <v>27</v>
       </c>
-      <c r="B28" s="9"/>
-      <c r="C28" s="9" t="s">
+      <c r="B28" s="6"/>
+      <c r="C28" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="30" ht="14.25">
-      <c r="A30" s="7" t="s">
+      <c r="A30" s="3" t="s">
         <v>28</v>
       </c>
-      <c r="B30" s="5"/>
-      <c r="C30" s="5"/>
+      <c r="B30" s="3"/>
+      <c r="C30" s="3"/>
     </row>
     <row r="31" ht="14.25">
-      <c r="A31" s="9" t="s">
+      <c r="A31" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B31" s="9" t="s">
+      <c r="B31" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="C31" s="9" t="s">
+      <c r="C31" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="32" ht="14.25">
-      <c r="A32" s="9" t="s">
+      <c r="A32" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B32" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="C32" s="9" t="s">
+      <c r="B32" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C32" s="6" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="33" ht="14.25">
-      <c r="A33" s="9" t="s">
+      <c r="A33" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B33" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="C33" s="9" t="s">
+      <c r="B33" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C33" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="34" ht="14.25">
-      <c r="A34" s="9" t="s">
+      <c r="A34" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B34" s="9"/>
-      <c r="C34" s="9" t="s">
+      <c r="B34" s="6"/>
+      <c r="C34" s="6" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="35" ht="14.25">
-      <c r="A35" s="9" t="s">
+      <c r="A35" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B35" s="9"/>
-      <c r="C35" s="9" t="s">
+      <c r="B35" s="6"/>
+      <c r="C35" s="6" t="s">
         <v>16</v>
       </c>
     </row>
     <row r="36" ht="14.25">
-      <c r="A36" s="9" t="s">
+      <c r="A36" s="6" t="s">
         <v>17</v>
       </c>
-      <c r="B36" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="C36" s="9" t="s">
+      <c r="B36" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C36" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="37" ht="14.25">
-      <c r="A37" s="9" t="s">
+      <c r="A37" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="B37" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="C37" s="9" t="s">
+      <c r="B37" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C37" s="6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="38" ht="14.25">
+      <c r="A38" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B38" s="6"/>
+      <c r="C38" s="6" t="s">
         <v>6</v>
       </c>
     </row>
     <row r="39" ht="14.25">
-      <c r="A39" s="11" t="s">
-        <v>30</v>
-      </c>
-      <c r="B39" s="12"/>
-      <c r="C39" s="12"/>
+      <c r="A39" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="B39" s="6"/>
+      <c r="C39" s="6" t="s">
+        <v>6</v>
+      </c>
     </row>
     <row r="40" ht="14.25">
-      <c r="A40" s="9" t="s">
+      <c r="A40" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B40" s="6"/>
+      <c r="C40" s="6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="41" ht="14.25">
+      <c r="A41" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="B41" s="6"/>
+      <c r="C41" s="6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="43" ht="14.25">
+      <c r="A43" s="7" t="s">
+        <v>34</v>
+      </c>
+      <c r="B43" s="7"/>
+      <c r="C43" s="7"/>
+    </row>
+    <row r="44" ht="14.25">
+      <c r="A44" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B40" s="9" t="s">
+      <c r="B44" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="C40" s="9" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="41" ht="14.25">
-      <c r="A41" s="9" t="s">
+      <c r="C44" s="6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="45" ht="14.25">
+      <c r="A45" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B41" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="C41" s="9" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="42" ht="14.25">
-      <c r="A42" s="9" t="s">
+      <c r="B45" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C45" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="46" ht="14.25">
+      <c r="A46" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B42" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="C42" s="9" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="43" ht="14.25">
-      <c r="A43" s="9" t="s">
+      <c r="B46" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C46" s="6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="47" ht="14.25">
+      <c r="A47" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B43" s="9"/>
-      <c r="C43" s="9" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="44" ht="14.25">
-      <c r="A44" s="9" t="s">
+      <c r="B47" s="6"/>
+      <c r="C47" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="48" ht="14.25">
+      <c r="A48" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B44" s="9"/>
-      <c r="C44" s="9" t="s">
+      <c r="B48" s="6"/>
+      <c r="C48" s="6" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="45" ht="14.25">
-      <c r="A45" s="9" t="s">
-        <v>31</v>
-      </c>
-      <c r="B45" s="9"/>
-      <c r="C45" s="9" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="46" ht="14.25">
-      <c r="A46" s="9" t="s">
+    <row r="49" ht="14.25">
+      <c r="A49" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="B49" s="6"/>
+      <c r="C49" s="6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="50" ht="14.25">
+      <c r="A50" s="6" t="s">
         <v>29</v>
       </c>
-      <c r="B46" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="C46" s="9" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="48" ht="14.25">
-      <c r="A48" s="7" t="s">
-        <v>32</v>
-      </c>
-      <c r="B48" s="5"/>
-      <c r="C48" s="5"/>
-    </row>
-    <row r="49" ht="14.25">
-      <c r="A49" s="9" t="s">
+      <c r="B50" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C50" s="6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="52" ht="14.25">
+      <c r="A52" s="3" t="s">
+        <v>36</v>
+      </c>
+      <c r="B52" s="3"/>
+      <c r="C52" s="3"/>
+    </row>
+    <row r="53" ht="14.25">
+      <c r="A53" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="B49" s="9" t="s">
+      <c r="B53" s="6" t="s">
         <v>5</v>
       </c>
-      <c r="C49" s="9" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="50" ht="14.25">
-      <c r="A50" s="9" t="s">
+      <c r="C53" s="6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="54" ht="14.25">
+      <c r="A54" s="6" t="s">
         <v>14</v>
       </c>
-      <c r="B50" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="C50" s="9" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="51" ht="14.25">
-      <c r="A51" s="9" t="s">
+      <c r="B54" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C54" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="55" ht="14.25">
+      <c r="A55" s="6" t="s">
         <v>11</v>
       </c>
-      <c r="B51" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="C51" s="9" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="52" ht="14.25">
-      <c r="A52" s="9" t="s">
+      <c r="B55" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C55" s="6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="56" ht="14.25">
+      <c r="A56" s="6" t="s">
         <v>12</v>
       </c>
-      <c r="B52" s="9"/>
-      <c r="C52" s="9" t="s">
-        <v>13</v>
-      </c>
-    </row>
-    <row r="53" ht="14.25">
-      <c r="A53" s="9" t="s">
+      <c r="B56" s="6"/>
+      <c r="C56" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="57" ht="14.25">
+      <c r="A57" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="B53" s="9"/>
-      <c r="C53" s="9" t="s">
+      <c r="B57" s="6"/>
+      <c r="C57" s="6" t="s">
         <v>16</v>
       </c>
     </row>
-    <row r="54" ht="14.25">
-      <c r="A54" s="9" t="s">
-        <v>33</v>
-      </c>
-      <c r="B54" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="C54" s="9" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="55" ht="14.25">
-      <c r="A55" s="10" t="s">
-        <v>34</v>
-      </c>
-      <c r="B55" s="9" t="s">
-        <v>8</v>
-      </c>
-      <c r="C55" s="9" t="s">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="56" ht="14.25">
-      <c r="A56" s="9" t="s">
-        <v>35</v>
-      </c>
-      <c r="B56" s="9"/>
-      <c r="C56" s="9" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="57" ht="14.25">
-      <c r="A57" s="9" t="s">
+    <row r="58" ht="14.25">
+      <c r="A58" s="6" t="s">
         <v>37</v>
       </c>
-      <c r="B57" s="9"/>
-      <c r="C57" s="9" t="s">
-        <v>6</v>
+      <c r="B58" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C58" s="6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="59" ht="14.25">
+      <c r="A59" s="6" t="s">
+        <v>38</v>
+      </c>
+      <c r="B59" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C59" s="6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="60" ht="14.25">
+      <c r="A60" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="B60" s="6"/>
+      <c r="C60" s="6" t="s">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="61" ht="14.25">
+      <c r="A61" s="6" t="s">
+        <v>41</v>
+      </c>
+      <c r="B61" s="6"/>
+      <c r="C61" s="6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="63" ht="14.25">
+      <c r="A63" s="8" t="s">
+        <v>42</v>
+      </c>
+      <c r="B63" s="3"/>
+      <c r="C63" s="3"/>
+    </row>
+    <row r="64" ht="14.25">
+      <c r="A64" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B64" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C64" s="6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="65" ht="14.25">
+      <c r="A65" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B65" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C65" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="66" ht="14.25">
+      <c r="A66" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B66" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C66" s="6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="67" ht="14.25">
+      <c r="A67" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B67" s="6"/>
+      <c r="C67" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="68" ht="14.25">
+      <c r="A68" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B68" s="6"/>
+      <c r="C68" s="6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="69" ht="14.25">
+      <c r="A69" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B69" s="6"/>
+      <c r="C69" s="6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="71" ht="14.25">
+      <c r="A71" s="9" t="s">
+        <v>43</v>
+      </c>
+      <c r="B71" s="7"/>
+      <c r="C71" s="7"/>
+    </row>
+    <row r="72" ht="14.25">
+      <c r="A72" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B72" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C72" s="6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="73" ht="14.25">
+      <c r="A73" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B73" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C73" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="74" ht="14.25">
+      <c r="A74" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B74" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C74" s="6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="75" ht="14.25">
+      <c r="A75" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B75" s="6"/>
+      <c r="C75" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="76" ht="14.25">
+      <c r="A76" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B76" s="6"/>
+      <c r="C76" s="6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="77" ht="14.25">
+      <c r="A77" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B77" s="6"/>
+      <c r="C77" s="6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="79" ht="14.25">
+      <c r="A79" s="9" t="s">
+        <v>44</v>
+      </c>
+      <c r="B79" s="7"/>
+      <c r="C79" s="7"/>
+    </row>
+    <row r="80" ht="14.25">
+      <c r="A80" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B80" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C80" s="6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="81" ht="14.25">
+      <c r="A81" s="6" t="s">
+        <v>14</v>
+      </c>
+      <c r="B81" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C81" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="82" ht="14.25">
+      <c r="A82" s="6" t="s">
+        <v>11</v>
+      </c>
+      <c r="B82" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="C82" s="6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="83" ht="14.25">
+      <c r="A83" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B83" s="6"/>
+      <c r="C83" s="6" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="84" ht="14.25">
+      <c r="A84" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="B84" s="6"/>
+      <c r="C84" s="6" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="85" ht="14.25">
+      <c r="A85" s="6" t="s">
+        <v>25</v>
+      </c>
+      <c r="B85" s="6"/>
+      <c r="C85" s="6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="87" ht="14.25">
+      <c r="A87" s="10" t="s">
+        <v>45</v>
+      </c>
+      <c r="B87" s="11"/>
+      <c r="C87" s="11"/>
+    </row>
+    <row r="88" ht="14.25">
+      <c r="A88" s="6" t="s">
+        <v>4</v>
+      </c>
+      <c r="B88" s="6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C88" s="6" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="89" ht="14.25">
+      <c r="A89" s="6" t="s">
+        <v>12</v>
+      </c>
+      <c r="B89" s="6"/>
+      <c r="C89" s="6" t="s">
+        <v>13</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="13">
+  <mergeCells count="17">
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="F1:H1"/>
     <mergeCell ref="A3:C3"/>
@@ -1363,8 +1650,12 @@
     <mergeCell ref="F19:H19"/>
     <mergeCell ref="A20:C20"/>
     <mergeCell ref="A30:C30"/>
-    <mergeCell ref="A39:C39"/>
-    <mergeCell ref="A48:C48"/>
+    <mergeCell ref="A43:C43"/>
+    <mergeCell ref="A52:C52"/>
+    <mergeCell ref="A63:C63"/>
+    <mergeCell ref="A71:C71"/>
+    <mergeCell ref="A79:C79"/>
+    <mergeCell ref="A87:C87"/>
   </mergeCells>
   <printOptions headings="0" gridLines="0"/>
   <pageMargins left="0.69999999999999996" right="0.69999999999999996" top="0.75" bottom="0.75" header="0.29999999999999999" footer="0.29999999999999999"/>

</xml_diff>